<commit_message>
new robo key and renaming the files
</commit_message>
<xml_diff>
--- a/data/robo_sensor_key.xlsx
+++ b/data/robo_sensor_key.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/graceleuchtenberger/Library/Mobile Documents/com~apple~CloudDocs/Documents/Density_field/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD392255-7DA0-7B4C-9A26-8DCA6D9F0EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D06F226-49CE-6548-AF63-F75301708BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6420" yWindow="2580" windowWidth="28040" windowHeight="17440" xr2:uid="{E5551131-2787-2048-A137-0E9CDA1D5CCA}"/>
+    <workbookView xWindow="1360" yWindow="680" windowWidth="28040" windowHeight="17160" xr2:uid="{E5551131-2787-2048-A137-0E9CDA1D5CCA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -862,7 +862,7 @@
         <v>13</v>
       </c>
       <c r="B16">
-        <v>29</v>
+        <v>98</v>
       </c>
       <c r="C16">
         <v>1</v>

</xml_diff>

<commit_message>
we're getting silly with it
</commit_message>
<xml_diff>
--- a/data/robo_sensor_key.xlsx
+++ b/data/robo_sensor_key.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/graceleuchtenberger/Library/Mobile Documents/com~apple~CloudDocs/Documents/Density_field/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D06F226-49CE-6548-AF63-F75301708BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7C11D1-863E-8347-B3FA-9507CF924CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1360" yWindow="680" windowWidth="28040" windowHeight="17160" xr2:uid="{E5551131-2787-2048-A137-0E9CDA1D5CCA}"/>
   </bookViews>
@@ -589,7 +589,7 @@
         <v>94</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="s">
         <v>26</v>
@@ -681,7 +681,7 @@
         <v>97</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" t="s">
         <v>26</v>
@@ -750,7 +750,7 @@
         <v>99</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" t="s">
         <v>26</v>
@@ -796,7 +796,7 @@
         <v>27</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" t="s">
         <v>26</v>
@@ -862,10 +862,10 @@
         <v>13</v>
       </c>
       <c r="B16">
-        <v>98</v>
+        <v>29</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="s">
         <v>26</v>
@@ -957,7 +957,7 @@
         <v>44</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" t="s">
         <v>26</v>

</xml_diff>